<commit_message>
12/9 - saturday calss end
</commit_message>
<xml_diff>
--- a/Excel/Excel Class.xlsx
+++ b/Excel/Excel Class.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\devid\Desktop\PW\DA-Aug-Batch-PW\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DE0B896-C7B7-4583-AFAE-95D62A0DF4DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9B180B1-B652-4B16-8E2F-87B2D4078A29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Basic" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,8 @@
     <sheet name="Shortcuts" sheetId="2" r:id="rId3"/>
     <sheet name="Exercise" sheetId="4" r:id="rId4"/>
     <sheet name="Basic Functions" sheetId="5" r:id="rId5"/>
+    <sheet name="Text functions" sheetId="6" r:id="rId6"/>
+    <sheet name="Date Time functions" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -78,7 +80,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -100,7 +102,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="277">
   <si>
     <t>Navigate between sheets</t>
   </si>
@@ -558,16 +560,694 @@
       <t>)</t>
     </r>
   </si>
+  <si>
+    <t>average for numbers in range that meet the condition</t>
+  </si>
+  <si>
+    <t>Logical Functions</t>
+  </si>
+  <si>
+    <r>
+      <t>IFS(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="4" tint="0.39997558519241921"/>
+        <rFont val="Rockwell"/>
+        <family val="1"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A2&gt;90, "A",</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Rockwell"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="7" tint="-0.249977111117893"/>
+        <rFont val="Rockwell"/>
+        <family val="1"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A2&gt; 80, "B"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Rockwell"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Rockwell"/>
+        <family val="1"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">A2&gt; 70, "C", </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="6" tint="-0.249977111117893"/>
+        <rFont val="Rockwell"/>
+        <family val="1"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>TRUE, "Fail"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Rockwell"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> )</t>
+    </r>
+  </si>
+  <si>
+    <t>functions that return TRUE or FALSE</t>
+  </si>
+  <si>
+    <t>AND</t>
+  </si>
+  <si>
+    <t>OR</t>
+  </si>
+  <si>
+    <t>invert karo</t>
+  </si>
+  <si>
+    <t>NOT()</t>
+  </si>
+  <si>
+    <t>Truth Tables</t>
+  </si>
+  <si>
+    <t>one input</t>
+  </si>
+  <si>
+    <t>two inputs - Both conditions should be TRUE</t>
+  </si>
+  <si>
+    <t>two inputs - One of the conditions should be TRUE</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>y</t>
+  </si>
+  <si>
+    <t>" + "</t>
+  </si>
+  <si>
+    <t>" * "</t>
+  </si>
+  <si>
+    <t>AND(condition1, condition2)</t>
+  </si>
+  <si>
+    <t>OR(condition1, condition2)</t>
+  </si>
+  <si>
+    <t>Only those people with attendence higher than 90 and marks higher than 80</t>
+  </si>
+  <si>
+    <t>AND is giving TRUE when both conditions are TRUE</t>
+  </si>
+  <si>
+    <t>if any condition is false, then it will return FALSE</t>
+  </si>
+  <si>
+    <t>marks</t>
+  </si>
+  <si>
+    <t>subject</t>
+  </si>
+  <si>
+    <t>physics</t>
+  </si>
+  <si>
+    <t>biology</t>
+  </si>
+  <si>
+    <t>drawing</t>
+  </si>
+  <si>
+    <t>coding</t>
+  </si>
+  <si>
+    <t>maths</t>
+  </si>
+  <si>
+    <t>Eligiblity</t>
+  </si>
+  <si>
+    <t>Text Functions</t>
+  </si>
+  <si>
+    <t>are used to clean or transform or format</t>
+  </si>
+  <si>
+    <t>join two string (text/words)</t>
+  </si>
+  <si>
+    <t>CONCAT:</t>
+  </si>
+  <si>
+    <t>Hello</t>
+  </si>
+  <si>
+    <t>without delimiters - space, comma</t>
+  </si>
+  <si>
+    <t>function</t>
+  </si>
+  <si>
+    <t>joins two strings, with a delimiter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&amp; </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ampersand - joins text as it is</t>
+  </si>
+  <si>
+    <t>TEXTJOIN:</t>
+  </si>
+  <si>
+    <t>concatenate</t>
+  </si>
+  <si>
+    <t>LEFT</t>
+  </si>
+  <si>
+    <t>RIGHT</t>
+  </si>
+  <si>
+    <t>MID</t>
+  </si>
+  <si>
+    <t>LEN</t>
+  </si>
+  <si>
+    <t>TRIM</t>
+  </si>
+  <si>
+    <t>Excel Tips</t>
+  </si>
+  <si>
+    <t xml:space="preserve">extract characters from start </t>
+  </si>
+  <si>
+    <t>ACB-1223-US</t>
+  </si>
+  <si>
+    <t>extracts from the middle</t>
+  </si>
+  <si>
+    <t>dfg-1223-US</t>
+  </si>
+  <si>
+    <t>hth-1223-US</t>
+  </si>
+  <si>
+    <t>fdg-3454-US</t>
+  </si>
+  <si>
+    <t>dsa-1223-US</t>
+  </si>
+  <si>
+    <t>extracts from the end</t>
+  </si>
+  <si>
+    <t>data.xlsx</t>
+  </si>
+  <si>
+    <t>returns the number of characters in text</t>
+  </si>
+  <si>
+    <t>extra spaces removal</t>
+  </si>
+  <si>
+    <t>it leaves single space between words</t>
+  </si>
+  <si>
+    <t>!#Idr    ees</t>
+  </si>
+  <si>
+    <t xml:space="preserve">excel               tips     </t>
+  </si>
+  <si>
+    <t>UPPER()</t>
+  </si>
+  <si>
+    <t>LOWER()</t>
+  </si>
+  <si>
+    <t>PROPER()</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HellO IDrees </t>
+  </si>
+  <si>
+    <t>HellO Idrees</t>
+  </si>
+  <si>
+    <t>HellO IDrees</t>
+  </si>
+  <si>
+    <t>converts text into UPPERCASE</t>
+  </si>
+  <si>
+    <t>converts text into lowercase</t>
+  </si>
+  <si>
+    <t>capitalizes first letters</t>
+  </si>
+  <si>
+    <t>FIND()</t>
+  </si>
+  <si>
+    <t>returns position of character in text</t>
+  </si>
+  <si>
+    <t>if it does not find, throws VALUE error</t>
+  </si>
+  <si>
+    <t>case - sensetive</t>
+  </si>
+  <si>
+    <t>DATE TIME Functions</t>
+  </si>
+  <si>
+    <t>pattern of characters too</t>
+  </si>
+  <si>
+    <t>Date Functions</t>
+  </si>
+  <si>
+    <t>TODAY()</t>
+  </si>
+  <si>
+    <t>NOW()</t>
+  </si>
+  <si>
+    <t>DATE()</t>
+  </si>
+  <si>
+    <t>DATEDIF()</t>
+  </si>
+  <si>
+    <t>creates a date using - year, month, day</t>
+  </si>
+  <si>
+    <t>calculate difference between two dates</t>
+  </si>
+  <si>
+    <t>Excel stores dates as serial numbers</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>time</t>
+  </si>
+  <si>
+    <t>TODAY() gives the current Date</t>
+  </si>
+  <si>
+    <t>NOW() - gives current date time</t>
+  </si>
+  <si>
+    <t>dynamic - changes</t>
+  </si>
+  <si>
+    <t>static</t>
+  </si>
+  <si>
+    <t>Ctrl + ;</t>
+  </si>
+  <si>
+    <t>Ctrl + Shift + ;</t>
+  </si>
+  <si>
+    <t>Current Date - static</t>
+  </si>
+  <si>
+    <t>Current Time - static</t>
+  </si>
+  <si>
+    <t>TEXT(date, format)</t>
+  </si>
+  <si>
+    <t>formats a date in our given format</t>
+  </si>
+  <si>
+    <t>date - dd- mm- yyyy</t>
+  </si>
+  <si>
+    <t>TEXT(C40,"dd/mm/yyyy" )</t>
+  </si>
+  <si>
+    <t>mmm</t>
+  </si>
+  <si>
+    <t>Jan</t>
+  </si>
+  <si>
+    <t>dd- mmm- yyyy</t>
+  </si>
+  <si>
+    <t>dd- mmmm- yyyy</t>
+  </si>
+  <si>
+    <t>mmmm</t>
+  </si>
+  <si>
+    <t>January</t>
+  </si>
+  <si>
+    <t>dd</t>
+  </si>
+  <si>
+    <t>ddd</t>
+  </si>
+  <si>
+    <t>Wed</t>
+  </si>
+  <si>
+    <t>dddd</t>
+  </si>
+  <si>
+    <t>Wednesday</t>
+  </si>
+  <si>
+    <t>hh:mm:ss</t>
+  </si>
+  <si>
+    <t>return the current date - from our PC</t>
+  </si>
+  <si>
+    <t>returns current date and time - from our PC</t>
+  </si>
+  <si>
+    <t>HOUR()</t>
+  </si>
+  <si>
+    <t>MINUTE()</t>
+  </si>
+  <si>
+    <t>Day()</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EXAMPLE: </t>
+  </si>
+  <si>
+    <t>task a</t>
+  </si>
+  <si>
+    <t>task b</t>
+  </si>
+  <si>
+    <t>task c</t>
+  </si>
+  <si>
+    <t>task d</t>
+  </si>
+  <si>
+    <t>task e</t>
+  </si>
+  <si>
+    <t>Deadlines</t>
+  </si>
+  <si>
+    <t>Days Remaning</t>
+  </si>
+  <si>
+    <t>Deadline Calculator</t>
+  </si>
+  <si>
+    <t>D53 - TODAY()</t>
+  </si>
+  <si>
+    <t>Age Calculator</t>
+  </si>
+  <si>
+    <t>Hritik</t>
+  </si>
+  <si>
+    <t>Manab</t>
+  </si>
+  <si>
+    <t>Waseem</t>
+  </si>
+  <si>
+    <t>DOB</t>
+  </si>
+  <si>
+    <t>Age(years)</t>
+  </si>
+  <si>
+    <t>Datedif()</t>
+  </si>
+  <si>
+    <t>Datedif(start_date, end_date, unit)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">unit: </t>
+  </si>
+  <si>
+    <t>"D"</t>
+  </si>
+  <si>
+    <t>"M"</t>
+  </si>
+  <si>
+    <t>"YD"</t>
+  </si>
+  <si>
+    <t>"YM"</t>
+  </si>
+  <si>
+    <t>"MD"</t>
+  </si>
+  <si>
+    <t>"Y"</t>
+  </si>
+  <si>
+    <t>days between dates</t>
+  </si>
+  <si>
+    <t>months between</t>
+  </si>
+  <si>
+    <t>years between</t>
+  </si>
+  <si>
+    <t>diffence in days, ignoring months/years</t>
+  </si>
+  <si>
+    <t>diffence in months, ignoring days/years</t>
+  </si>
+  <si>
+    <t>differnce in days ignoring years</t>
+  </si>
+  <si>
+    <t>DATEDIF(D63,TODAY(), "Y")</t>
+  </si>
+  <si>
+    <t>Datedif(1/1/2026,"12/09/2026","D")</t>
+  </si>
+  <si>
+    <t>TEXT(TODAY(),"dddd, mmmm dd, yyyy")</t>
+  </si>
+  <si>
+    <t>TEXT(NOW(),"hh:mm:ss AM/PM</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="4"/>
+        <rFont val="Rockwell"/>
+        <family val="1"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"Today is "</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Rockwell"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">      </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="9"/>
+        <rFont val="Rockwell"/>
+        <family val="1"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">&amp; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Rockwell"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">     </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Rockwell"/>
+        <family val="1"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">TEXT(TODAY(),"dddd, mmmm dd, yyyy")    </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="9"/>
+        <rFont val="Rockwell"/>
+        <family val="1"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&amp;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Rockwell"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">     </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="4"/>
+        <rFont val="Rockwell"/>
+        <family val="1"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>" and the current time is "</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Rockwell"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">   </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="9"/>
+        <rFont val="Rockwell"/>
+        <family val="1"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &amp;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Rockwell"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Rockwell"/>
+        <family val="1"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>TEXT(NOW(),"hh:mm:ss AM/PM")</t>
+    </r>
+  </si>
+  <si>
+    <t>returns text/strings</t>
+  </si>
+  <si>
+    <t>WORKDAY(start_date, days, [holidays])</t>
+  </si>
+  <si>
+    <t>used to calculate a date that is a certain number of workdays</t>
+  </si>
+  <si>
+    <t>before or after a given date</t>
+  </si>
+  <si>
+    <t>workdays exclude Sunday, Saturday, or holiday which we can provide</t>
+  </si>
+  <si>
+    <t>workday after 10 days</t>
+  </si>
+  <si>
+    <t>WORKDAY(C94, 10, {"24/09/2026"})</t>
+  </si>
+  <si>
+    <t>24 is a holiday</t>
+  </si>
+  <si>
+    <t>28 is a holiday</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="_ [$₹-4009]\ * #,##0.00_ ;_ [$₹-4009]\ * \-#,##0.00_ ;_ [$₹-4009]\ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="165" formatCode="[$-14009]dd/mm/yyyy;@"/>
+    <numFmt numFmtId="167" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    <numFmt numFmtId="169" formatCode="[$-10409]hh:mm\ AM/PM;@"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -683,8 +1363,95 @@
       <family val="1"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="4"/>
+      <name val="Rockwell"/>
+      <family val="1"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="6" tint="-0.249977111117893"/>
+      <name val="Rockwell"/>
+      <family val="1"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Rockwell"/>
+      <family val="1"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Rockwell"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Rockwell"/>
+      <family val="1"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Rockwell"/>
+      <family val="1"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Rockwell"/>
+      <family val="1"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="9"/>
+      <name val="Rockwell"/>
+      <family val="1"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF188038"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="9"/>
+      <name val="Rockwell"/>
+      <family val="1"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Rockwell"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -721,8 +1488,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -756,12 +1541,36 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -803,6 +1612,48 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -831,70 +1682,112 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="22" fontId="22" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="22" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -928,8 +1821,8 @@
       <xdr:row>41</xdr:row>
       <xdr:rowOff>64284</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="121" name="Ink 120">
@@ -948,7 +1841,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="121" name="Ink 120">
@@ -1314,18 +2207,18 @@
       <c r="E1" s="6"/>
     </row>
     <row r="2" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="38" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
     </row>
     <row r="3" spans="2:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
+      <c r="B3" s="38"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="38"/>
     </row>
     <row r="4" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B4" s="5" t="s">
@@ -1419,18 +2312,18 @@
       </c>
     </row>
     <row r="14" spans="2:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="20" t="s">
+      <c r="B14" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
+      <c r="C14" s="38"/>
+      <c r="D14" s="38"/>
+      <c r="E14" s="38"/>
     </row>
     <row r="15" spans="2:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="20"/>
-      <c r="E15" s="20"/>
+      <c r="B15" s="38"/>
+      <c r="C15" s="38"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="38"/>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B16" s="5" t="s">
@@ -1471,7 +2364,7 @@
         <v>62</v>
       </c>
       <c r="D19" s="8">
-        <f t="shared" ref="D18:D23" si="1">C19 / $C$16</f>
+        <f t="shared" ref="D19:D23" si="1">C19 / $C$16</f>
         <v>0.62</v>
       </c>
     </row>
@@ -1524,34 +2417,34 @@
       </c>
     </row>
     <row r="26" spans="2:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="20" t="s">
+      <c r="B26" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="C26" s="20"/>
-      <c r="D26" s="20"/>
-      <c r="E26" s="20"/>
-      <c r="F26" s="20"/>
+      <c r="C26" s="38"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="38"/>
+      <c r="F26" s="38"/>
     </row>
     <row r="27" spans="2:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="20"/>
-      <c r="C27" s="20"/>
-      <c r="D27" s="20"/>
-      <c r="E27" s="20"/>
-      <c r="F27" s="20"/>
+      <c r="B27" s="38"/>
+      <c r="C27" s="38"/>
+      <c r="D27" s="38"/>
+      <c r="E27" s="38"/>
+      <c r="F27" s="38"/>
     </row>
     <row r="28" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="C28" s="19" t="s">
+      <c r="C28" s="37" t="s">
         <v>48</v>
       </c>
-      <c r="D28" s="19"/>
-      <c r="E28" s="19"/>
-      <c r="F28" s="19"/>
-      <c r="G28" s="19"/>
-      <c r="H28" s="19"/>
-      <c r="I28" s="19"/>
-      <c r="J28" s="19"/>
-      <c r="K28" s="19"/>
-      <c r="L28" s="19"/>
+      <c r="D28" s="37"/>
+      <c r="E28" s="37"/>
+      <c r="F28" s="37"/>
+      <c r="G28" s="37"/>
+      <c r="H28" s="37"/>
+      <c r="I28" s="37"/>
+      <c r="J28" s="37"/>
+      <c r="K28" s="37"/>
+      <c r="L28" s="37"/>
     </row>
     <row r="29" spans="2:12" x14ac:dyDescent="0.25">
       <c r="C29" s="9">
@@ -2053,7 +2946,7 @@
     <tabColor theme="7" tint="0.39997558519241921"/>
   </sheetPr>
   <dimension ref="B3:M22"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="8.796875" customWidth="1"/>
     <col min="4" max="4" width="9.69921875" customWidth="1"/>
@@ -2061,257 +2954,265 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:13" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22" t="s">
+      <c r="C3" s="40"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="22"/>
+      <c r="F3" s="40"/>
     </row>
     <row r="4" spans="2:13" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
-    </row>
-    <row r="5" spans="2:13" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="B5" s="24" t="s">
+      <c r="B4" s="40"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="40"/>
+      <c r="F4" s="40"/>
+    </row>
+    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B5" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="24"/>
-      <c r="D5" s="24"/>
-      <c r="E5" s="24" t="s">
+      <c r="C5" s="42"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="F5" s="24"/>
+      <c r="F5" s="42"/>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
     </row>
-    <row r="6" spans="2:13" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="B6" s="24" t="s">
+    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B6" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="24"/>
-      <c r="D6" s="24"/>
-      <c r="E6" s="24" t="s">
+      <c r="C6" s="42"/>
+      <c r="D6" s="42"/>
+      <c r="E6" s="42" t="s">
         <v>4</v>
       </c>
-      <c r="F6" s="24"/>
+      <c r="F6" s="42"/>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
     </row>
-    <row r="7" spans="2:13" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="B7" s="23" t="s">
+    <row r="7" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B7" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="23"/>
-      <c r="D7" s="23"/>
-      <c r="E7" s="24" t="s">
+      <c r="C7" s="41"/>
+      <c r="D7" s="41"/>
+      <c r="E7" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="F7" s="24"/>
+      <c r="F7" s="42"/>
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
     </row>
-    <row r="8" spans="2:13" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="B8" s="23"/>
-      <c r="C8" s="23"/>
-      <c r="D8" s="23"/>
-      <c r="E8" s="24"/>
-      <c r="F8" s="24"/>
-      <c r="I8" s="27" t="s">
+    <row r="8" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B8" s="41"/>
+      <c r="C8" s="41"/>
+      <c r="D8" s="41"/>
+      <c r="E8" s="42"/>
+      <c r="F8" s="42"/>
+      <c r="I8" s="45" t="s">
         <v>23</v>
       </c>
-      <c r="J8" s="27"/>
-      <c r="K8" s="27"/>
-      <c r="L8" s="27"/>
+      <c r="J8" s="45"/>
+      <c r="K8" s="45"/>
+      <c r="L8" s="45"/>
       <c r="M8" s="2"/>
     </row>
-    <row r="9" spans="2:13" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="B9" s="24" t="s">
+    <row r="9" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B9" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="24"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="24" t="s">
+      <c r="C9" s="42"/>
+      <c r="D9" s="42"/>
+      <c r="E9" s="42" t="s">
         <v>9</v>
       </c>
-      <c r="F9" s="24"/>
-      <c r="I9" s="27"/>
-      <c r="J9" s="27"/>
-      <c r="K9" s="27"/>
-      <c r="L9" s="27"/>
+      <c r="F9" s="42"/>
+      <c r="I9" s="45"/>
+      <c r="J9" s="45"/>
+      <c r="K9" s="45"/>
+      <c r="L9" s="45"/>
       <c r="M9" s="2"/>
     </row>
-    <row r="10" spans="2:13" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="B10" s="24" t="s">
+    <row r="10" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B10" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24" t="s">
+      <c r="C10" s="42"/>
+      <c r="D10" s="42"/>
+      <c r="E10" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="F10" s="24"/>
-      <c r="I10" s="27"/>
-      <c r="J10" s="27"/>
-      <c r="K10" s="27"/>
-      <c r="L10" s="27"/>
+      <c r="F10" s="42"/>
+      <c r="I10" s="45"/>
+      <c r="J10" s="45"/>
+      <c r="K10" s="45"/>
+      <c r="L10" s="45"/>
       <c r="M10" s="2"/>
     </row>
-    <row r="11" spans="2:13" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="B11" s="24" t="s">
+    <row r="11" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B11" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="24"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="26" t="s">
+      <c r="C11" s="42"/>
+      <c r="D11" s="42"/>
+      <c r="E11" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F11" s="26"/>
-      <c r="I11" s="27"/>
-      <c r="J11" s="27"/>
-      <c r="K11" s="27"/>
-      <c r="L11" s="27"/>
+      <c r="F11" s="44"/>
+      <c r="I11" s="45"/>
+      <c r="J11" s="45"/>
+      <c r="K11" s="45"/>
+      <c r="L11" s="45"/>
       <c r="M11" s="2"/>
     </row>
-    <row r="12" spans="2:13" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="B12" s="24" t="s">
+    <row r="12" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B12" s="42" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="24"/>
-      <c r="D12" s="24"/>
-      <c r="E12" s="26" t="s">
+      <c r="C12" s="42"/>
+      <c r="D12" s="42"/>
+      <c r="E12" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="F12" s="26"/>
-      <c r="I12" s="27"/>
-      <c r="J12" s="27"/>
-      <c r="K12" s="27"/>
-      <c r="L12" s="27"/>
+      <c r="F12" s="44"/>
+      <c r="I12" s="45"/>
+      <c r="J12" s="45"/>
+      <c r="K12" s="45"/>
+      <c r="L12" s="45"/>
       <c r="M12" s="2"/>
     </row>
-    <row r="13" spans="2:13" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="B13" s="26" t="s">
+    <row r="13" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B13" s="44" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="26"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26" t="s">
+      <c r="C13" s="44"/>
+      <c r="D13" s="44"/>
+      <c r="E13" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="F13" s="26"/>
-      <c r="I13" s="27"/>
-      <c r="J13" s="27"/>
-      <c r="K13" s="27"/>
-      <c r="L13" s="27"/>
+      <c r="F13" s="44"/>
+      <c r="I13" s="45"/>
+      <c r="J13" s="45"/>
+      <c r="K13" s="45"/>
+      <c r="L13" s="45"/>
       <c r="M13" s="2"/>
     </row>
-    <row r="14" spans="2:13" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="B14" s="25" t="s">
+    <row r="14" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B14" s="43" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="25"/>
-      <c r="D14" s="25"/>
-      <c r="E14" s="26" t="s">
+      <c r="C14" s="43"/>
+      <c r="D14" s="43"/>
+      <c r="E14" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="F14" s="26"/>
-      <c r="I14" s="27"/>
-      <c r="J14" s="27"/>
-      <c r="K14" s="27"/>
-      <c r="L14" s="27"/>
+      <c r="F14" s="44"/>
+      <c r="I14" s="45"/>
+      <c r="J14" s="45"/>
+      <c r="K14" s="45"/>
+      <c r="L14" s="45"/>
       <c r="M14" s="2"/>
     </row>
-    <row r="15" spans="2:13" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="B15" s="25"/>
-      <c r="C15" s="25"/>
-      <c r="D15" s="25"/>
-      <c r="E15" s="26"/>
-      <c r="F15" s="26"/>
-      <c r="I15" s="27"/>
-      <c r="J15" s="27"/>
-      <c r="K15" s="27"/>
-      <c r="L15" s="27"/>
+    <row r="15" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B15" s="43"/>
+      <c r="C15" s="43"/>
+      <c r="D15" s="43"/>
+      <c r="E15" s="44"/>
+      <c r="F15" s="44"/>
+      <c r="I15" s="45"/>
+      <c r="J15" s="45"/>
+      <c r="K15" s="45"/>
+      <c r="L15" s="45"/>
       <c r="M15" s="2"/>
     </row>
-    <row r="16" spans="2:13" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="B16" s="26" t="s">
+    <row r="16" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B16" s="44" t="s">
         <v>37</v>
       </c>
-      <c r="C16" s="26"/>
-      <c r="D16" s="26"/>
-      <c r="E16" s="26" t="s">
+      <c r="C16" s="44"/>
+      <c r="D16" s="44"/>
+      <c r="E16" s="44" t="s">
         <v>38</v>
       </c>
-      <c r="F16" s="26"/>
+      <c r="F16" s="44"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
       <c r="M16" s="2"/>
     </row>
-    <row r="17" spans="2:13" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="B17" s="26" t="s">
+    <row r="17" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B17" s="44" t="s">
         <v>54</v>
       </c>
-      <c r="C17" s="26"/>
-      <c r="D17" s="26"/>
-      <c r="E17" s="26" t="s">
+      <c r="C17" s="44"/>
+      <c r="D17" s="44"/>
+      <c r="E17" s="44" t="s">
         <v>53</v>
       </c>
-      <c r="F17" s="26"/>
+      <c r="F17" s="44"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
       <c r="L17" s="2"/>
       <c r="M17" s="2"/>
     </row>
-    <row r="18" spans="2:13" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="B18" s="26" t="s">
+    <row r="18" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B18" s="44" t="s">
         <v>82</v>
       </c>
-      <c r="C18" s="26"/>
-      <c r="D18" s="26"/>
-      <c r="E18" s="26" t="s">
+      <c r="C18" s="44"/>
+      <c r="D18" s="44"/>
+      <c r="E18" s="44" t="s">
         <v>81</v>
       </c>
-      <c r="F18" s="26"/>
-    </row>
-    <row r="19" spans="2:13" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="B19" s="21"/>
-      <c r="C19" s="21"/>
-      <c r="D19" s="21"/>
-      <c r="E19" s="21"/>
-      <c r="F19" s="21"/>
-    </row>
-    <row r="20" spans="2:13" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="B20" s="21"/>
-      <c r="C20" s="21"/>
-      <c r="D20" s="21"/>
-      <c r="E20" s="21"/>
-      <c r="F20" s="21"/>
-    </row>
-    <row r="21" spans="2:13" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="B21" s="21"/>
-      <c r="C21" s="21"/>
-      <c r="D21" s="21"/>
-      <c r="E21" s="21"/>
-      <c r="F21" s="21"/>
-    </row>
-    <row r="22" spans="2:13" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="F18" s="44"/>
+    </row>
+    <row r="19" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B19" s="44" t="s">
+        <v>209</v>
+      </c>
+      <c r="C19" s="44"/>
+      <c r="D19" s="44"/>
+      <c r="E19" s="44" t="s">
+        <v>207</v>
+      </c>
+      <c r="F19" s="44"/>
+    </row>
+    <row r="20" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B20" s="44" t="s">
+        <v>210</v>
+      </c>
+      <c r="C20" s="44"/>
+      <c r="D20" s="44"/>
+      <c r="E20" s="44" t="s">
+        <v>208</v>
+      </c>
+      <c r="F20" s="44"/>
+    </row>
+    <row r="21" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B21" s="39"/>
+      <c r="C21" s="39"/>
+      <c r="D21" s="39"/>
+      <c r="E21" s="39"/>
+      <c r="F21" s="39"/>
+    </row>
+    <row r="22" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
@@ -2325,12 +3226,12 @@
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="E6:F6"/>
+    <mergeCell ref="E13:F13"/>
     <mergeCell ref="B21:D21"/>
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="B16:D16"/>
-    <mergeCell ref="E13:F13"/>
     <mergeCell ref="B17:D17"/>
     <mergeCell ref="B18:D18"/>
     <mergeCell ref="B19:D19"/>
@@ -2604,7 +3505,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF72FC96-74E6-469B-BE37-9240C49DD4A1}">
-  <dimension ref="A3:S56"/>
+  <dimension ref="A3:S122"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="8.796875" customWidth="1"/>
@@ -2616,25 +3517,25 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:15" ht="18" x14ac:dyDescent="0.35">
-      <c r="B3" s="31" t="s">
+      <c r="B3" s="47" t="s">
         <v>66</v>
       </c>
-      <c r="C3" s="31"/>
+      <c r="C3" s="47"/>
     </row>
     <row r="4" spans="2:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>67</v>
       </c>
-      <c r="K4" s="33" t="s">
+      <c r="K4" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="L4" s="32" t="s">
+      <c r="L4" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="M4" s="32" t="s">
+      <c r="M4" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="N4" s="34" t="s">
+      <c r="N4" s="22" t="s">
         <v>71</v>
       </c>
     </row>
@@ -2715,11 +3616,11 @@
       </c>
     </row>
     <row r="10" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="C10" s="29" t="s">
+      <c r="C10" s="48" t="s">
         <v>70</v>
       </c>
-      <c r="D10" s="29"/>
-      <c r="E10" s="29"/>
+      <c r="D10" s="48"/>
+      <c r="E10" s="48"/>
       <c r="F10">
         <f>SUM(1,2,3)</f>
         <v>6</v>
@@ -2783,10 +3684,10 @@
       </c>
     </row>
     <row r="14" spans="2:15" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B14" s="35" t="s">
+      <c r="B14" s="49" t="s">
         <v>72</v>
       </c>
-      <c r="C14" s="35"/>
+      <c r="C14" s="49"/>
     </row>
     <row r="15" spans="2:15" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
@@ -2794,7 +3695,7 @@
       </c>
     </row>
     <row r="16" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="F16" s="30"/>
+      <c r="F16" s="19"/>
       <c r="M16" t="s">
         <v>74</v>
       </c>
@@ -2803,244 +3704,246 @@
       </c>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="F17" s="41" t="s">
+      <c r="F17" s="25" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="18" spans="1:19" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B18" s="39" t="s">
+      <c r="B18" s="53" t="s">
         <v>78</v>
       </c>
-      <c r="C18" s="39"/>
-      <c r="D18" s="39"/>
-      <c r="E18" s="36" t="s">
+      <c r="C18" s="53"/>
+      <c r="D18" s="53"/>
+      <c r="E18" s="50" t="s">
         <v>79</v>
       </c>
-      <c r="F18" s="36"/>
-      <c r="G18" s="36"/>
-      <c r="H18" s="36"/>
-      <c r="I18" s="36"/>
-      <c r="J18" s="28" t="s">
+      <c r="F18" s="50"/>
+      <c r="G18" s="50"/>
+      <c r="H18" s="50"/>
+      <c r="I18" s="50"/>
+      <c r="J18" s="46" t="s">
         <v>80</v>
       </c>
-      <c r="K18" s="28"/>
+      <c r="K18" s="46"/>
     </row>
     <row r="19" spans="1:19" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B19" s="39" t="s">
+      <c r="B19" s="53" t="s">
         <v>77</v>
       </c>
-      <c r="C19" s="39"/>
-      <c r="D19" s="39"/>
-      <c r="E19" s="36" t="s">
+      <c r="C19" s="53"/>
+      <c r="D19" s="53"/>
+      <c r="E19" s="50" t="s">
         <v>76</v>
       </c>
-      <c r="F19" s="36"/>
-      <c r="G19" s="36"/>
-      <c r="H19" s="36"/>
-      <c r="I19" s="36"/>
-      <c r="J19" s="28">
+      <c r="F19" s="50"/>
+      <c r="G19" s="50"/>
+      <c r="H19" s="50"/>
+      <c r="I19" s="50"/>
+      <c r="J19" s="46">
         <f>SUM(N5:N12)</f>
         <v>235</v>
       </c>
-      <c r="K19" s="28"/>
-    </row>
-    <row r="20" spans="1:19" s="41" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B20" s="39" t="s">
+      <c r="K19" s="46"/>
+    </row>
+    <row r="20" spans="1:19" s="25" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B20" s="53" t="s">
         <v>89</v>
       </c>
-      <c r="C20" s="39"/>
-      <c r="D20" s="39"/>
-      <c r="E20" s="36" t="s">
+      <c r="C20" s="53"/>
+      <c r="D20" s="53"/>
+      <c r="E20" s="50" t="s">
         <v>90</v>
       </c>
-      <c r="F20" s="36"/>
-      <c r="G20" s="36"/>
-      <c r="H20" s="36"/>
-      <c r="I20" s="36"/>
-      <c r="J20" s="28">
+      <c r="F20" s="50"/>
+      <c r="G20" s="50"/>
+      <c r="H20" s="50"/>
+      <c r="I20" s="50"/>
+      <c r="J20" s="46">
         <f>PRODUCT(N6:N10)</f>
         <v>10125000</v>
       </c>
-      <c r="K20" s="28"/>
+      <c r="K20" s="46"/>
     </row>
     <row r="21" spans="1:19" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B21" s="39" t="s">
+      <c r="B21" s="53" t="s">
         <v>84</v>
       </c>
-      <c r="C21" s="39"/>
-      <c r="D21" s="39"/>
-      <c r="E21" s="36" t="s">
+      <c r="C21" s="53"/>
+      <c r="D21" s="53"/>
+      <c r="E21" s="50" t="s">
         <v>83</v>
       </c>
-      <c r="F21" s="36"/>
-      <c r="G21" s="36"/>
-      <c r="H21" s="36"/>
-      <c r="I21" s="36"/>
-      <c r="J21" s="28">
+      <c r="F21" s="50"/>
+      <c r="G21" s="50"/>
+      <c r="H21" s="50"/>
+      <c r="I21" s="50"/>
+      <c r="J21" s="46">
         <f xml:space="preserve"> SUMIF(N5:N12, "&gt;20")</f>
         <v>205</v>
       </c>
-      <c r="K21" s="28"/>
+      <c r="K21" s="46"/>
     </row>
     <row r="22" spans="1:19" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B22" s="39" t="s">
+      <c r="B22" s="53" t="s">
         <v>85</v>
       </c>
-      <c r="C22" s="39"/>
-      <c r="D22" s="39"/>
-      <c r="E22" s="37" t="s">
+      <c r="C22" s="53"/>
+      <c r="D22" s="53"/>
+      <c r="E22" s="52" t="s">
         <v>88</v>
       </c>
-      <c r="F22" s="37"/>
-      <c r="G22" s="37"/>
-      <c r="H22" s="37"/>
-      <c r="I22" s="37"/>
-      <c r="J22" s="28">
+      <c r="F22" s="52"/>
+      <c r="G22" s="52"/>
+      <c r="H22" s="52"/>
+      <c r="I22" s="52"/>
+      <c r="J22" s="46">
         <f>SUMPRODUCT(P30:P33,Q30:Q33)</f>
         <v>2250</v>
       </c>
-      <c r="K22" s="28"/>
+      <c r="K22" s="46"/>
     </row>
     <row r="23" spans="1:19" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A23" s="41"/>
-      <c r="B23" s="39" t="s">
+      <c r="A23" s="25"/>
+      <c r="B23" s="53" t="s">
         <v>91</v>
       </c>
-      <c r="C23" s="39"/>
-      <c r="D23" s="39"/>
-      <c r="E23" s="21"/>
-      <c r="F23" s="21"/>
-      <c r="G23" s="21"/>
-      <c r="H23" s="21"/>
-      <c r="I23" s="21"/>
-      <c r="J23" s="28">
+      <c r="C23" s="53"/>
+      <c r="D23" s="53"/>
+      <c r="E23" s="39"/>
+      <c r="F23" s="39"/>
+      <c r="G23" s="39"/>
+      <c r="H23" s="39"/>
+      <c r="I23" s="39"/>
+      <c r="J23" s="46">
         <f>AVERAGE(N5:N12)</f>
         <v>29.375</v>
       </c>
-      <c r="K23" s="28"/>
+      <c r="K23" s="46"/>
     </row>
     <row r="24" spans="1:19" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B24" s="39" t="s">
+      <c r="B24" s="53" t="s">
         <v>92</v>
       </c>
-      <c r="C24" s="39"/>
-      <c r="D24" s="39"/>
-      <c r="E24" s="21"/>
-      <c r="F24" s="21"/>
-      <c r="G24" s="21"/>
-      <c r="H24" s="21"/>
-      <c r="I24" s="21"/>
-      <c r="J24" s="28">
+      <c r="C24" s="53"/>
+      <c r="D24" s="53"/>
+      <c r="E24" s="56" t="s">
+        <v>117</v>
+      </c>
+      <c r="F24" s="56"/>
+      <c r="G24" s="56"/>
+      <c r="H24" s="56"/>
+      <c r="I24" s="56"/>
+      <c r="J24" s="46">
         <f>AVERAGEIF(N5:N12,"&gt;10")</f>
         <v>32.142857142857146</v>
       </c>
-      <c r="K24" s="28"/>
+      <c r="K24" s="46"/>
       <c r="P24">
         <v>2</v>
       </c>
       <c r="Q24">
         <v>3</v>
       </c>
-      <c r="R24" s="38">
+      <c r="R24" s="23">
         <f>PRODUCT(P24:Q24)</f>
         <v>6</v>
       </c>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B25" s="48" t="s">
+      <c r="B25" s="54" t="s">
         <v>93</v>
       </c>
-      <c r="C25" s="48"/>
-      <c r="D25" s="48"/>
-      <c r="E25" s="21"/>
-      <c r="F25" s="21"/>
-      <c r="G25" s="21"/>
-      <c r="H25" s="21"/>
-      <c r="I25" s="21"/>
-      <c r="J25" s="28">
+      <c r="C25" s="54"/>
+      <c r="D25" s="54"/>
+      <c r="E25" s="39"/>
+      <c r="F25" s="39"/>
+      <c r="G25" s="39"/>
+      <c r="H25" s="39"/>
+      <c r="I25" s="39"/>
+      <c r="J25" s="46">
         <f>AVERAGEIFS(N5:N12, L5:L12,"&gt;75")</f>
         <v>32.5</v>
       </c>
-      <c r="K25" s="28"/>
+      <c r="K25" s="46"/>
       <c r="P25">
         <v>2</v>
       </c>
       <c r="Q25">
         <v>3</v>
       </c>
-      <c r="R25" s="38">
+      <c r="R25" s="23">
         <f t="shared" ref="R25:R27" si="0">PRODUCT(P25:Q25)</f>
         <v>6</v>
       </c>
     </row>
-    <row r="26" spans="1:19" s="41" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B26" s="49" t="s">
+    <row r="26" spans="1:19" s="25" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B26" s="55" t="s">
         <v>95</v>
       </c>
-      <c r="C26" s="49"/>
-      <c r="D26" s="49"/>
-      <c r="E26" s="21" t="s">
+      <c r="C26" s="55"/>
+      <c r="D26" s="55"/>
+      <c r="E26" s="39" t="s">
         <v>102</v>
       </c>
-      <c r="F26" s="21"/>
-      <c r="G26" s="21"/>
-      <c r="H26" s="21"/>
-      <c r="I26" s="21"/>
-      <c r="J26" s="28">
+      <c r="F26" s="39"/>
+      <c r="G26" s="39"/>
+      <c r="H26" s="39"/>
+      <c r="I26" s="39"/>
+      <c r="J26" s="46">
         <f>COUNT(E20:I28)</f>
         <v>0</v>
       </c>
-      <c r="K26" s="28"/>
-      <c r="R26" s="47"/>
+      <c r="K26" s="46"/>
+      <c r="R26" s="30"/>
     </row>
     <row r="27" spans="1:19" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B27" s="49" t="s">
+      <c r="B27" s="55" t="s">
         <v>100</v>
       </c>
-      <c r="C27" s="49"/>
-      <c r="D27" s="49"/>
-      <c r="E27" s="21" t="s">
+      <c r="C27" s="55"/>
+      <c r="D27" s="55"/>
+      <c r="E27" s="39" t="s">
         <v>101</v>
       </c>
-      <c r="F27" s="21"/>
-      <c r="G27" s="21"/>
-      <c r="H27" s="21"/>
-      <c r="I27" s="21"/>
-      <c r="J27" s="28">
+      <c r="F27" s="39"/>
+      <c r="G27" s="39"/>
+      <c r="H27" s="39"/>
+      <c r="I27" s="39"/>
+      <c r="J27" s="46">
         <f>COUNTA(E20:I28)</f>
-        <v>6</v>
-      </c>
-      <c r="K27" s="28"/>
+        <v>7</v>
+      </c>
+      <c r="K27" s="46"/>
       <c r="P27">
         <v>2</v>
       </c>
       <c r="Q27">
         <v>3</v>
       </c>
-      <c r="R27" s="38">
+      <c r="R27" s="23">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
     </row>
     <row r="28" spans="1:19" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B28" s="49" t="s">
+      <c r="B28" s="55" t="s">
         <v>97</v>
       </c>
-      <c r="C28" s="49"/>
-      <c r="D28" s="49"/>
-      <c r="E28" s="21" t="s">
+      <c r="C28" s="55"/>
+      <c r="D28" s="55"/>
+      <c r="E28" s="39" t="s">
         <v>99</v>
       </c>
-      <c r="F28" s="21"/>
-      <c r="G28" s="21"/>
-      <c r="H28" s="21"/>
-      <c r="I28" s="21"/>
-      <c r="J28" s="28">
+      <c r="F28" s="39"/>
+      <c r="G28" s="39"/>
+      <c r="H28" s="39"/>
+      <c r="I28" s="39"/>
+      <c r="J28" s="46">
         <f>COUNTBLANK(O28:O33)</f>
         <v>2</v>
       </c>
-      <c r="K28" s="28"/>
-      <c r="R28" s="38">
+      <c r="K28" s="46"/>
+      <c r="R28" s="23">
         <f>SUM(R24:R27)</f>
         <v>18</v>
       </c>
@@ -3050,21 +3953,21 @@
       </c>
     </row>
     <row r="29" spans="1:19" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B29" s="49" t="s">
+      <c r="B29" s="55" t="s">
         <v>96</v>
       </c>
-      <c r="C29" s="49"/>
-      <c r="D29" s="49"/>
-      <c r="E29" s="21"/>
-      <c r="F29" s="21"/>
-      <c r="G29" s="21"/>
-      <c r="H29" s="21"/>
-      <c r="I29" s="21"/>
-      <c r="J29" s="28">
+      <c r="C29" s="55"/>
+      <c r="D29" s="55"/>
+      <c r="E29" s="39"/>
+      <c r="F29" s="39"/>
+      <c r="G29" s="39"/>
+      <c r="H29" s="39"/>
+      <c r="I29" s="39"/>
+      <c r="J29" s="46">
         <f xml:space="preserve"> COUNTIF(L5:L12, "&gt;70")</f>
         <v>4</v>
       </c>
-      <c r="K29" s="28"/>
+      <c r="K29" s="46"/>
       <c r="P29" s="11" t="s">
         <v>34</v>
       </c>
@@ -3073,22 +3976,22 @@
       </c>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B30" s="50" t="s">
+      <c r="B30" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="C30" s="50"/>
-      <c r="D30" s="50"/>
-      <c r="E30" s="21"/>
-      <c r="F30" s="21"/>
-      <c r="G30" s="21"/>
-      <c r="H30" s="21"/>
-      <c r="I30" s="21"/>
-      <c r="J30" s="28">
+      <c r="C30" s="51"/>
+      <c r="D30" s="51"/>
+      <c r="E30" s="39"/>
+      <c r="F30" s="39"/>
+      <c r="G30" s="39"/>
+      <c r="H30" s="39"/>
+      <c r="I30" s="39"/>
+      <c r="J30" s="46">
         <f xml:space="preserve"> COUNTIFS(L5:L12, "&gt;70", N5:N12, "&gt;10")</f>
         <v>4</v>
       </c>
-      <c r="K30" s="28"/>
-      <c r="O30" s="41" t="s">
+      <c r="K30" s="46"/>
+      <c r="O30" s="25" t="s">
         <v>29</v>
       </c>
       <c r="P30">
@@ -3103,22 +4006,22 @@
       </c>
     </row>
     <row r="31" spans="1:19" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B31" s="49" t="s">
+      <c r="B31" s="55" t="s">
         <v>103</v>
       </c>
-      <c r="C31" s="49"/>
-      <c r="D31" s="49"/>
-      <c r="E31" s="21"/>
-      <c r="F31" s="21"/>
-      <c r="G31" s="21"/>
-      <c r="H31" s="21"/>
-      <c r="I31" s="21"/>
-      <c r="J31" s="28">
+      <c r="C31" s="55"/>
+      <c r="D31" s="55"/>
+      <c r="E31" s="39"/>
+      <c r="F31" s="39"/>
+      <c r="G31" s="39"/>
+      <c r="H31" s="39"/>
+      <c r="I31" s="39"/>
+      <c r="J31" s="46">
         <f>MIN(N5:N12)</f>
         <v>10</v>
       </c>
-      <c r="K31" s="28"/>
-      <c r="O31" s="41" t="s">
+      <c r="K31" s="46"/>
+      <c r="O31" s="25" t="s">
         <v>30</v>
       </c>
       <c r="P31">
@@ -3133,22 +4036,22 @@
       </c>
     </row>
     <row r="32" spans="1:19" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B32" s="49" t="s">
+      <c r="B32" s="55" t="s">
         <v>104</v>
       </c>
-      <c r="C32" s="49"/>
-      <c r="D32" s="49"/>
-      <c r="E32" s="21"/>
-      <c r="F32" s="21"/>
-      <c r="G32" s="21"/>
-      <c r="H32" s="21"/>
-      <c r="I32" s="21"/>
-      <c r="J32" s="28">
+      <c r="C32" s="55"/>
+      <c r="D32" s="55"/>
+      <c r="E32" s="39"/>
+      <c r="F32" s="39"/>
+      <c r="G32" s="39"/>
+      <c r="H32" s="39"/>
+      <c r="I32" s="39"/>
+      <c r="J32" s="46">
         <f>MAX(N5:N12)</f>
         <v>45</v>
       </c>
-      <c r="K32" s="28"/>
-      <c r="O32" s="41" t="s">
+      <c r="K32" s="46"/>
+      <c r="O32" s="25" t="s">
         <v>31</v>
       </c>
       <c r="P32">
@@ -3163,7 +4066,7 @@
       </c>
     </row>
     <row r="33" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="O33" s="41" t="s">
+      <c r="O33" s="25" t="s">
         <v>32</v>
       </c>
       <c r="P33">
@@ -3184,7 +4087,7 @@
       <c r="F34" t="s">
         <v>105</v>
       </c>
-      <c r="Q34" s="40" t="s">
+      <c r="Q34" s="24" t="s">
         <v>86</v>
       </c>
       <c r="R34">
@@ -3221,10 +4124,10 @@
     </row>
     <row r="41" spans="2:18" ht="14.4" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="42" spans="2:18" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B42" s="51" t="s">
+      <c r="B42" s="57" t="s">
         <v>94</v>
       </c>
-      <c r="C42" s="52"/>
+      <c r="C42" s="58"/>
     </row>
     <row r="43" spans="2:18" x14ac:dyDescent="0.25">
       <c r="C43" t="s">
@@ -3235,19 +4138,19 @@
       <c r="C45" t="s">
         <v>110</v>
       </c>
-      <c r="I45" s="45" t="s">
+      <c r="I45" s="66" t="s">
         <v>24</v>
       </c>
-      <c r="J45" s="44" t="s">
+      <c r="J45" s="28" t="s">
         <v>63</v>
       </c>
-      <c r="K45" s="44" t="s">
+      <c r="K45" s="28" t="s">
         <v>64</v>
       </c>
-      <c r="L45" s="46" t="s">
+      <c r="L45" s="29" t="s">
         <v>71</v>
       </c>
-      <c r="M45" s="46" t="s">
+      <c r="M45" s="29" t="s">
         <v>113</v>
       </c>
       <c r="N45" t="s">
@@ -3255,16 +4158,16 @@
       </c>
     </row>
     <row r="46" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="I46" s="41" t="s">
+      <c r="I46" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="J46" s="43">
+      <c r="J46" s="27">
         <v>96</v>
       </c>
-      <c r="K46" s="43">
+      <c r="K46" s="27">
         <v>95</v>
       </c>
-      <c r="L46" s="42">
+      <c r="L46" s="26">
         <v>30</v>
       </c>
       <c r="N46" t="str" cm="1">
@@ -3276,191 +4179,578 @@
       <c r="C47" t="s">
         <v>109</v>
       </c>
-      <c r="D47" s="53" t="s">
+      <c r="D47" s="31" t="s">
         <v>111</v>
       </c>
-      <c r="E47" s="53" t="s">
+      <c r="E47" s="31" t="s">
         <v>112</v>
       </c>
-      <c r="I47" s="41" t="s">
+      <c r="I47" s="25" t="s">
         <v>57</v>
       </c>
-      <c r="J47" s="43">
+      <c r="J47" s="27">
         <v>88</v>
       </c>
-      <c r="K47" s="43">
+      <c r="K47" s="27">
         <v>92</v>
       </c>
-      <c r="L47" s="42">
+      <c r="L47" s="26">
         <v>25</v>
       </c>
-      <c r="N47" s="41" t="str" cm="1">
+      <c r="N47" s="25" t="str" cm="1">
         <f t="array" ref="N47">_xlfn.IFS(K47 &gt; 90,"A", K47&gt;80, "B", K47&gt;70, "C",TRUE, "Needs Improvement" )</f>
         <v>A</v>
       </c>
     </row>
     <row r="48" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="D48" s="42">
+      <c r="D48" s="26">
         <v>18</v>
       </c>
-      <c r="E48" s="42" t="str">
+      <c r="E48" s="26" t="str">
         <f>IF(D48 &gt;= 18, "Voter", "Non-Voter")</f>
         <v>Voter</v>
       </c>
-      <c r="I48" s="41" t="s">
+      <c r="I48" s="25" t="s">
         <v>58</v>
       </c>
-      <c r="J48" s="43">
+      <c r="J48" s="27">
         <v>62</v>
       </c>
-      <c r="K48" s="43">
+      <c r="K48" s="27">
         <v>86</v>
       </c>
-      <c r="L48" s="42">
+      <c r="L48" s="26">
         <v>30</v>
       </c>
-      <c r="N48" s="41" t="str" cm="1">
+      <c r="N48" s="25" t="str" cm="1">
         <f t="array" ref="N48">_xlfn.IFS(K48 &gt; 90,"A", K48&gt;80, "B", K48&gt;70, "C",TRUE, "Needs Improvement" )</f>
         <v>B</v>
       </c>
     </row>
-    <row r="49" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="D49" s="42">
+    <row r="49" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="D49" s="26">
         <v>20</v>
       </c>
-      <c r="E49" s="42" t="str">
+      <c r="E49" s="26" t="str">
         <f t="shared" ref="E49:E53" si="2">IF(D49 &gt;= 18, "Voter", "Non-Voter")</f>
         <v>Voter</v>
       </c>
-      <c r="I49" s="41" t="s">
+      <c r="I49" s="25" t="s">
         <v>59</v>
       </c>
-      <c r="J49" s="43">
+      <c r="J49" s="27">
         <v>43</v>
       </c>
-      <c r="K49" s="43">
+      <c r="K49" s="27">
         <v>72</v>
       </c>
-      <c r="L49" s="42">
+      <c r="L49" s="26">
         <v>45</v>
       </c>
-      <c r="N49" s="41" t="str" cm="1">
+      <c r="N49" s="25" t="str" cm="1">
         <f t="array" ref="N49">_xlfn.IFS(K49 &gt; 90,"A", K49&gt;80, "B", K49&gt;70, "C",TRUE, "Needs Improvement" )</f>
         <v>C</v>
       </c>
     </row>
-    <row r="50" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="D50" s="42">
+    <row r="50" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="D50" s="26">
         <v>34</v>
       </c>
-      <c r="E50" s="42" t="str">
+      <c r="E50" s="26" t="str">
         <f t="shared" si="2"/>
         <v>Voter</v>
       </c>
-      <c r="I50" s="41" t="s">
+      <c r="I50" s="25" t="s">
         <v>60</v>
       </c>
-      <c r="J50" s="43">
+      <c r="J50" s="27">
         <v>87</v>
       </c>
-      <c r="K50" s="43">
+      <c r="K50" s="27">
         <v>88</v>
       </c>
-      <c r="L50" s="42">
+      <c r="L50" s="26">
         <v>30</v>
       </c>
-      <c r="N50" s="41" t="str" cm="1">
+      <c r="N50" s="25" t="str" cm="1">
         <f t="array" ref="N50">_xlfn.IFS(K50 &gt; 90,"A", K50&gt;80, "B", K50&gt;70, "C",TRUE, "Needs Improvement" )</f>
         <v>B</v>
       </c>
     </row>
-    <row r="51" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="D51" s="42">
+    <row r="51" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="D51" s="26">
         <v>6</v>
       </c>
-      <c r="E51" s="42" t="str">
+      <c r="E51" s="26" t="str">
         <f t="shared" si="2"/>
         <v>Non-Voter</v>
       </c>
-      <c r="I51" s="41" t="s">
+      <c r="I51" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="J51" s="43">
+      <c r="J51" s="27">
         <v>23</v>
       </c>
-      <c r="K51" s="43">
+      <c r="K51" s="27">
         <v>34</v>
       </c>
-      <c r="L51" s="42">
+      <c r="L51" s="26">
         <v>10</v>
       </c>
-      <c r="N51" s="41" t="str" cm="1">
+      <c r="N51" s="25" t="str" cm="1">
         <f t="array" ref="N51">_xlfn.IFS(K51 &gt; 90,"A", K51&gt;80, "B", K51&gt;70, "C",TRUE, "Needs Improvement" )</f>
         <v>Needs Improvement</v>
       </c>
     </row>
-    <row r="52" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="D52" s="42">
+    <row r="52" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="D52" s="26">
         <v>10</v>
       </c>
-      <c r="E52" s="42" t="str">
+      <c r="E52" s="26" t="str">
         <f t="shared" si="2"/>
         <v>Non-Voter</v>
       </c>
-      <c r="I52" s="41" t="s">
+      <c r="I52" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="J52" s="43">
+      <c r="J52" s="27">
         <v>97</v>
       </c>
-      <c r="K52" s="43">
+      <c r="K52" s="27">
         <v>41</v>
       </c>
-      <c r="L52" s="42">
+      <c r="L52" s="26">
         <v>45</v>
       </c>
-      <c r="N52" s="41" t="str" cm="1">
+      <c r="N52" s="25" t="str" cm="1">
         <f t="array" ref="N52">_xlfn.IFS(K52 &gt; 90,"A", K52&gt;80, "B", K52&gt;70, "C",TRUE, "Needs Improvement" )</f>
         <v>Needs Improvement</v>
       </c>
     </row>
-    <row r="53" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="D53" s="42">
+    <row r="53" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="D53" s="26">
         <v>55</v>
       </c>
-      <c r="E53" s="42" t="str">
+      <c r="E53" s="26" t="str">
         <f t="shared" si="2"/>
         <v>Voter</v>
       </c>
-      <c r="I53" s="41" t="s">
+      <c r="I53" s="25" t="s">
         <v>65</v>
       </c>
-      <c r="J53" s="43">
+      <c r="J53" s="27">
         <v>42</v>
       </c>
-      <c r="K53" s="43">
+      <c r="K53" s="27">
         <v>32</v>
       </c>
-      <c r="L53" s="42">
+      <c r="L53" s="26">
         <v>20</v>
       </c>
-      <c r="N53" s="41" t="str" cm="1">
+      <c r="N53" s="25" t="str" cm="1">
         <f t="array" ref="N53">_xlfn.IFS(K53 &gt; 90,"A", K53&gt;80, "B", K53&gt;70, "C",TRUE, "Needs Improvement" )</f>
         <v>Needs Improvement</v>
       </c>
     </row>
-    <row r="55" spans="3:14" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:14" x14ac:dyDescent="0.25">
       <c r="C55" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="56" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="C56" s="54" t="s">
+    <row r="56" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="C56" s="32" t="s">
         <v>116</v>
       </c>
     </row>
+    <row r="57" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="C57" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="60" spans="2:14" ht="14.4" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="61" spans="2:14" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B61" s="57" t="s">
+        <v>118</v>
+      </c>
+      <c r="C61" s="58"/>
+    </row>
+    <row r="62" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B62" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="63" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="D63" s="34">
+        <v>1</v>
+      </c>
+      <c r="E63" s="34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="2:14" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B66" s="59" t="s">
+        <v>124</v>
+      </c>
+      <c r="E66" t="s">
+        <v>123</v>
+      </c>
+      <c r="G66" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="67" spans="2:14" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B67" s="59" t="s">
+        <v>133</v>
+      </c>
+      <c r="E67" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="68" spans="2:14" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B68" s="59" t="s">
+        <v>134</v>
+      </c>
+      <c r="E68" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="70" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="C70" s="46" t="s">
+        <v>125</v>
+      </c>
+      <c r="D70" s="46"/>
+      <c r="E70" s="46"/>
+    </row>
+    <row r="71" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B71" s="60" t="s">
+        <v>129</v>
+      </c>
+      <c r="C71" s="60" t="s">
+        <v>130</v>
+      </c>
+      <c r="D71" s="61" t="s">
+        <v>122</v>
+      </c>
+      <c r="E71" s="62" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="72" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B72" s="63">
+        <v>0</v>
+      </c>
+      <c r="C72" s="63">
+        <v>0</v>
+      </c>
+      <c r="D72" s="64" t="b">
+        <f xml:space="preserve"> OR(B72,C72)</f>
+        <v>0</v>
+      </c>
+      <c r="E72" s="64" t="b">
+        <f xml:space="preserve"> AND(B72,C72)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B73" s="63">
+        <v>0</v>
+      </c>
+      <c r="C73" s="63">
+        <v>1</v>
+      </c>
+      <c r="D73" s="65" t="b">
+        <f t="shared" ref="D73:D75" si="3" xml:space="preserve"> OR(B73,C73)</f>
+        <v>1</v>
+      </c>
+      <c r="E73" s="64" t="b">
+        <f t="shared" ref="E73:E75" si="4" xml:space="preserve"> AND(B73,C73)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="2:14" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B74" s="63">
+        <v>1</v>
+      </c>
+      <c r="C74" s="63">
+        <v>0</v>
+      </c>
+      <c r="D74" s="65" t="b">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="E74" s="64" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="K74" s="66" t="s">
+        <v>24</v>
+      </c>
+      <c r="L74" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="M74" s="28" t="s">
+        <v>64</v>
+      </c>
+      <c r="N74" s="29" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="75" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B75" s="63">
+        <v>1</v>
+      </c>
+      <c r="C75" s="63">
+        <v>1</v>
+      </c>
+      <c r="D75" s="65" t="b">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="E75" s="65" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="K75" s="35" t="s">
+        <v>56</v>
+      </c>
+      <c r="L75" s="33">
+        <v>96</v>
+      </c>
+      <c r="M75" s="33">
+        <v>95</v>
+      </c>
+      <c r="N75" s="34">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="76" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="D76" s="34" t="s">
+        <v>131</v>
+      </c>
+      <c r="E76" s="34" t="s">
+        <v>132</v>
+      </c>
+      <c r="K76" s="35" t="s">
+        <v>57</v>
+      </c>
+      <c r="L76" s="33">
+        <v>88</v>
+      </c>
+      <c r="M76" s="33">
+        <v>92</v>
+      </c>
+      <c r="N76" s="34">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="77" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="K77" s="35" t="s">
+        <v>58</v>
+      </c>
+      <c r="L77" s="33">
+        <v>62</v>
+      </c>
+      <c r="M77" s="33">
+        <v>86</v>
+      </c>
+      <c r="N77" s="34">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="78" spans="2:14" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B78" s="68" t="s">
+        <v>138</v>
+      </c>
+      <c r="C78" s="68" t="s">
+        <v>139</v>
+      </c>
+      <c r="D78" s="59"/>
+      <c r="E78" s="59" t="s">
+        <v>145</v>
+      </c>
+      <c r="K78" s="35" t="s">
+        <v>59</v>
+      </c>
+      <c r="L78" s="33">
+        <v>43</v>
+      </c>
+      <c r="M78" s="33">
+        <v>72</v>
+      </c>
+      <c r="N78" s="34">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="79" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B79" s="67">
+        <v>75</v>
+      </c>
+      <c r="C79" s="67" t="s">
+        <v>140</v>
+      </c>
+      <c r="D79" t="b">
+        <f>AND(B79 &gt; 60, C79 = "physics")</f>
+        <v>1</v>
+      </c>
+      <c r="E79" t="str">
+        <f xml:space="preserve"> IF(AND(B79 &gt; 60, C79 = "physics"), "Eligible","Not Eligible")</f>
+        <v>Eligible</v>
+      </c>
+      <c r="K79" s="35" t="s">
+        <v>60</v>
+      </c>
+      <c r="L79" s="33">
+        <v>87</v>
+      </c>
+      <c r="M79" s="33">
+        <v>88</v>
+      </c>
+      <c r="N79" s="34">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="80" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B80" s="67">
+        <v>65</v>
+      </c>
+      <c r="C80" s="67" t="s">
+        <v>141</v>
+      </c>
+      <c r="D80" s="35" t="b">
+        <f t="shared" ref="D80:D84" si="5">AND(B80 &gt; 60, C80 = "physics")</f>
+        <v>0</v>
+      </c>
+      <c r="E80" s="35" t="str">
+        <f t="shared" ref="E80:E84" si="6">IF(AND(B80 &gt; 60, C80 = "physics"), "Eligible","Not Eligible")</f>
+        <v>Not Eligible</v>
+      </c>
+      <c r="K80" s="35" t="s">
+        <v>61</v>
+      </c>
+      <c r="L80" s="33">
+        <v>23</v>
+      </c>
+      <c r="M80" s="33">
+        <v>34</v>
+      </c>
+      <c r="N80" s="34">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="81" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B81" s="67">
+        <v>45</v>
+      </c>
+      <c r="C81" s="67" t="s">
+        <v>142</v>
+      </c>
+      <c r="D81" s="35" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="E81" s="35" t="str">
+        <f t="shared" si="6"/>
+        <v>Not Eligible</v>
+      </c>
+      <c r="K81" s="35" t="s">
+        <v>62</v>
+      </c>
+      <c r="L81" s="33">
+        <v>97</v>
+      </c>
+      <c r="M81" s="33">
+        <v>41</v>
+      </c>
+      <c r="N81" s="34">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="82" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B82" s="67">
+        <v>75</v>
+      </c>
+      <c r="C82" s="67" t="s">
+        <v>143</v>
+      </c>
+      <c r="D82" s="35" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="E82" s="35" t="str">
+        <f t="shared" si="6"/>
+        <v>Not Eligible</v>
+      </c>
+      <c r="K82" s="35" t="s">
+        <v>65</v>
+      </c>
+      <c r="L82" s="33">
+        <v>42</v>
+      </c>
+      <c r="M82" s="33">
+        <v>32</v>
+      </c>
+      <c r="N82" s="34">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="83" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B83" s="67">
+        <v>95</v>
+      </c>
+      <c r="C83" s="67" t="s">
+        <v>140</v>
+      </c>
+      <c r="D83" s="35" t="b">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="E83" s="35" t="str">
+        <f t="shared" si="6"/>
+        <v>Eligible</v>
+      </c>
+      <c r="K83" s="35"/>
+      <c r="L83" s="35"/>
+      <c r="M83" s="35"/>
+      <c r="N83" s="35"/>
+    </row>
+    <row r="84" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B84" s="67">
+        <v>25</v>
+      </c>
+      <c r="C84" s="67" t="s">
+        <v>144</v>
+      </c>
+      <c r="D84" s="35" t="b">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="E84" s="35" t="str">
+        <f t="shared" si="6"/>
+        <v>Not Eligible</v>
+      </c>
+      <c r="K84" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="86" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="K86" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="87" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="K87" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="122" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B122" t="s">
+        <v>191</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="49">
+  <mergeCells count="51">
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="C70:E70"/>
     <mergeCell ref="B42:C42"/>
     <mergeCell ref="B26:D26"/>
     <mergeCell ref="E26:I26"/>
@@ -3469,39 +4759,35 @@
     <mergeCell ref="E30:I30"/>
     <mergeCell ref="E31:I31"/>
     <mergeCell ref="E32:I32"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J28:K28"/>
     <mergeCell ref="J29:K29"/>
     <mergeCell ref="J30:K30"/>
     <mergeCell ref="J31:K31"/>
     <mergeCell ref="J32:K32"/>
     <mergeCell ref="B31:D31"/>
     <mergeCell ref="B32:D32"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="E21:I21"/>
+    <mergeCell ref="E22:I22"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="B22:D22"/>
     <mergeCell ref="E23:I23"/>
     <mergeCell ref="E24:I24"/>
     <mergeCell ref="E25:I25"/>
     <mergeCell ref="E27:I27"/>
     <mergeCell ref="E28:I28"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="B20:D20"/>
-    <mergeCell ref="E20:I20"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="B24:D24"/>
-    <mergeCell ref="B25:D25"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="E21:I21"/>
-    <mergeCell ref="E22:I22"/>
     <mergeCell ref="J20:K20"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="C10:E10"/>
@@ -3510,6 +4796,10 @@
     <mergeCell ref="J18:K18"/>
     <mergeCell ref="E18:I18"/>
     <mergeCell ref="E19:I19"/>
+    <mergeCell ref="E20:I20"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B20:D20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -3517,4 +4807,1275 @@
     <ignoredError sqref="J20" formulaRange="1"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5ABF673-38D3-4308-95CA-4D53C3C12963}">
+  <dimension ref="B2:M31"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="2" spans="3:13" ht="14.4" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="3:13" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C3" s="57" t="s">
+        <v>146</v>
+      </c>
+      <c r="D3" s="58"/>
+    </row>
+    <row r="5" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="7" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="D7" t="s">
+        <v>157</v>
+      </c>
+      <c r="J7" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="8" spans="3:13" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D8" s="69" t="s">
+        <v>149</v>
+      </c>
+      <c r="E8" t="s">
+        <v>148</v>
+      </c>
+      <c r="J8" s="59" t="str">
+        <f>_xlfn.CONCAT(L8, M8)</f>
+        <v>HelloIdrees</v>
+      </c>
+      <c r="K8" s="59"/>
+      <c r="L8" s="59" t="s">
+        <v>150</v>
+      </c>
+      <c r="M8" s="59" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="9" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="D9" s="69"/>
+      <c r="E9" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="10" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="D10" s="69"/>
+    </row>
+    <row r="11" spans="3:13" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D11" s="69" t="s">
+        <v>156</v>
+      </c>
+      <c r="E11" t="s">
+        <v>153</v>
+      </c>
+      <c r="J11" t="str">
+        <f>_xlfn.TEXTJOIN(" ", TRUE, L11,M11)</f>
+        <v>Hello Idrees</v>
+      </c>
+      <c r="L11" s="59" t="s">
+        <v>150</v>
+      </c>
+      <c r="M11" s="59" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="12" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="D12" s="69"/>
+    </row>
+    <row r="13" spans="3:13" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="D13" s="69" t="s">
+        <v>154</v>
+      </c>
+      <c r="E13" s="35" t="s">
+        <v>155</v>
+      </c>
+      <c r="J13" t="str">
+        <f xml:space="preserve"> L13 &amp; " " &amp; M13</f>
+        <v>Hello Idrees</v>
+      </c>
+      <c r="L13" s="59" t="s">
+        <v>150</v>
+      </c>
+      <c r="M13" s="59" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="15" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="F15" t="str">
+        <f xml:space="preserve"> "Hello" &amp; "Idrees"</f>
+        <v>HelloIdrees</v>
+      </c>
+    </row>
+    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>163</v>
+      </c>
+      <c r="D17" t="s">
+        <v>158</v>
+      </c>
+      <c r="E17" s="70" t="s">
+        <v>164</v>
+      </c>
+      <c r="H17" s="34" t="str">
+        <f>LEFT(B17, 5)</f>
+        <v>Excel</v>
+      </c>
+    </row>
+    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>165</v>
+      </c>
+      <c r="D18" t="s">
+        <v>160</v>
+      </c>
+      <c r="E18" s="70" t="s">
+        <v>166</v>
+      </c>
+      <c r="H18" s="34" t="str">
+        <f>MID(B18, 5, 4)</f>
+        <v>1223</v>
+      </c>
+      <c r="K18" s="35" t="s">
+        <v>165</v>
+      </c>
+      <c r="L18" s="35" t="str">
+        <f>MID(K18,5,4)</f>
+        <v>1223</v>
+      </c>
+    </row>
+    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B19" s="35" t="s">
+        <v>172</v>
+      </c>
+      <c r="D19" t="s">
+        <v>159</v>
+      </c>
+      <c r="E19" s="70" t="s">
+        <v>171</v>
+      </c>
+      <c r="H19" s="34" t="str">
+        <f>RIGHT(B19,4)</f>
+        <v>xlsx</v>
+      </c>
+      <c r="K19" s="35" t="s">
+        <v>167</v>
+      </c>
+      <c r="L19" s="35" t="str">
+        <f>MID(K19,5,4)</f>
+        <v>1223</v>
+      </c>
+    </row>
+    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="H20" s="34"/>
+      <c r="K20" s="35" t="s">
+        <v>169</v>
+      </c>
+      <c r="L20" s="35" t="str">
+        <f>MID(K20,5,4)</f>
+        <v>3454</v>
+      </c>
+    </row>
+    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B21" s="71" t="s">
+        <v>176</v>
+      </c>
+      <c r="D21" t="s">
+        <v>161</v>
+      </c>
+      <c r="E21" s="70" t="s">
+        <v>173</v>
+      </c>
+      <c r="H21" s="34">
+        <f>LEN(B21)</f>
+        <v>12</v>
+      </c>
+      <c r="K21" s="35" t="s">
+        <v>168</v>
+      </c>
+      <c r="L21" s="35" t="str">
+        <f>MID(K21,5,4)</f>
+        <v>1223</v>
+      </c>
+    </row>
+    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
+        <v>177</v>
+      </c>
+      <c r="D22" t="s">
+        <v>162</v>
+      </c>
+      <c r="E22" s="70" t="s">
+        <v>174</v>
+      </c>
+      <c r="H22" s="34" t="str">
+        <f xml:space="preserve"> TRIM(B22)</f>
+        <v>excel tips</v>
+      </c>
+      <c r="K22" s="35" t="s">
+        <v>170</v>
+      </c>
+      <c r="L22" s="35" t="str">
+        <f>MID(K22,5,4)</f>
+        <v>1223</v>
+      </c>
+    </row>
+    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="E23" s="70" t="s">
+        <v>175</v>
+      </c>
+      <c r="K23" s="35" t="s">
+        <v>165</v>
+      </c>
+      <c r="L23" s="35" t="str">
+        <f>MID(K23,5,4)</f>
+        <v>1223</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
+        <v>183</v>
+      </c>
+      <c r="D25" t="s">
+        <v>178</v>
+      </c>
+      <c r="E25" s="70" t="s">
+        <v>184</v>
+      </c>
+      <c r="H25" t="str">
+        <f>UPPER(B25)</f>
+        <v>HELLO IDREES</v>
+      </c>
+    </row>
+    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B26" s="35" t="s">
+        <v>181</v>
+      </c>
+      <c r="D26" t="s">
+        <v>179</v>
+      </c>
+      <c r="E26" s="70" t="s">
+        <v>185</v>
+      </c>
+      <c r="H26" t="str">
+        <f>LOWER(B26)</f>
+        <v xml:space="preserve">hello idrees </v>
+      </c>
+    </row>
+    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B27" t="s">
+        <v>182</v>
+      </c>
+      <c r="D27" t="s">
+        <v>180</v>
+      </c>
+      <c r="E27" s="70" t="s">
+        <v>186</v>
+      </c>
+      <c r="H27" t="str">
+        <f>PROPER(B27)</f>
+        <v>Hello Idrees</v>
+      </c>
+    </row>
+    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B28" s="35" t="s">
+        <v>182</v>
+      </c>
+      <c r="D28" t="s">
+        <v>187</v>
+      </c>
+      <c r="E28" s="70" t="s">
+        <v>188</v>
+      </c>
+      <c r="H28">
+        <f>FIND("s", B28)</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="E29" s="70" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="E30" s="70" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="E31" s="70" t="s">
+        <v>192</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C3:D3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3669CD76-13DF-47AC-A8EF-04D36B174787}">
+  <dimension ref="B3:I109"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="20.796875" customWidth="1"/>
+    <col min="4" max="4" width="17.796875" customWidth="1"/>
+    <col min="5" max="5" width="18.19921875" customWidth="1"/>
+    <col min="6" max="6" width="19.796875" customWidth="1"/>
+    <col min="7" max="7" width="14.19921875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B3" s="72" t="s">
+        <v>193</v>
+      </c>
+      <c r="C3" s="72"/>
+      <c r="D3" s="72"/>
+      <c r="E3" s="72"/>
+    </row>
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B4" s="72"/>
+      <c r="C4" s="72"/>
+      <c r="D4" s="72"/>
+      <c r="E4" s="72"/>
+    </row>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>194</v>
+      </c>
+      <c r="D6" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>195</v>
+      </c>
+      <c r="D7" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C8" t="s">
+        <v>196</v>
+      </c>
+      <c r="D8" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C9" t="s">
+        <v>197</v>
+      </c>
+      <c r="D9" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B15" s="34" t="s">
+        <v>201</v>
+      </c>
+      <c r="C15" s="34"/>
+      <c r="D15" s="34"/>
+      <c r="E15" s="34" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B16" s="33">
+        <v>1</v>
+      </c>
+      <c r="C16" s="73">
+        <v>1</v>
+      </c>
+      <c r="E16" s="34">
+        <v>0</v>
+      </c>
+      <c r="F16" s="75">
+        <v>0</v>
+      </c>
+      <c r="G16" s="77">
+        <v>0</v>
+      </c>
+      <c r="I16" s="81"/>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B17" s="33">
+        <v>2</v>
+      </c>
+      <c r="C17" s="73">
+        <v>2</v>
+      </c>
+      <c r="E17" s="34">
+        <v>0.1</v>
+      </c>
+      <c r="F17" s="75">
+        <v>0.1</v>
+      </c>
+      <c r="G17" s="77">
+        <v>0.1</v>
+      </c>
+      <c r="I17" s="81"/>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B18" s="33">
+        <v>3</v>
+      </c>
+      <c r="C18" s="73">
+        <v>3</v>
+      </c>
+      <c r="E18" s="78">
+        <v>0.2</v>
+      </c>
+      <c r="F18" s="75">
+        <v>0.19999999999999998</v>
+      </c>
+      <c r="G18" s="77">
+        <v>0.19999999999999998</v>
+      </c>
+      <c r="I18" s="81"/>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B19" s="33">
+        <v>4</v>
+      </c>
+      <c r="C19" s="73">
+        <v>4</v>
+      </c>
+      <c r="E19" s="34">
+        <v>0.5</v>
+      </c>
+      <c r="F19" s="75">
+        <v>0.5</v>
+      </c>
+      <c r="G19" s="77">
+        <v>0.5</v>
+      </c>
+      <c r="I19" s="81"/>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B20" s="33">
+        <v>46277</v>
+      </c>
+      <c r="C20" s="76">
+        <v>46277</v>
+      </c>
+      <c r="E20" s="34">
+        <v>0.625</v>
+      </c>
+      <c r="F20" s="75">
+        <v>0.625</v>
+      </c>
+      <c r="G20" s="77">
+        <v>0.625</v>
+      </c>
+      <c r="I20" s="81"/>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B21" s="33">
+        <v>46278</v>
+      </c>
+      <c r="C21" s="76">
+        <v>46278</v>
+      </c>
+      <c r="E21" s="78">
+        <v>0.75</v>
+      </c>
+      <c r="F21" s="75">
+        <v>0.75</v>
+      </c>
+      <c r="G21" s="77">
+        <v>0.75</v>
+      </c>
+      <c r="I21" s="81"/>
+    </row>
+    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B22" s="33">
+        <v>46279</v>
+      </c>
+      <c r="C22" s="76">
+        <v>46279</v>
+      </c>
+      <c r="E22" s="78">
+        <v>0.9</v>
+      </c>
+      <c r="F22" s="75">
+        <v>0.9</v>
+      </c>
+      <c r="G22" s="77">
+        <v>0.9</v>
+      </c>
+      <c r="I22" s="81"/>
+    </row>
+    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B23" s="33">
+        <v>46280</v>
+      </c>
+      <c r="C23" s="76">
+        <v>46280</v>
+      </c>
+      <c r="E23" s="78">
+        <v>0.95</v>
+      </c>
+      <c r="F23" s="75">
+        <v>0.95</v>
+      </c>
+      <c r="G23" s="77">
+        <v>0.95</v>
+      </c>
+      <c r="I23" s="81"/>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C24" s="76"/>
+      <c r="E24" s="74"/>
+    </row>
+    <row r="25" spans="2:9" ht="16.8" x14ac:dyDescent="0.4">
+      <c r="C25" s="80">
+        <v>45901</v>
+      </c>
+    </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C26" s="76"/>
+    </row>
+    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C27" s="76"/>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="E28" s="34" t="s">
+        <v>205</v>
+      </c>
+      <c r="F28" s="34"/>
+      <c r="G28" s="34" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="29" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B29" t="s">
+        <v>203</v>
+      </c>
+      <c r="E29" s="73">
+        <f ca="1" xml:space="preserve"> TODAY()</f>
+        <v>46277</v>
+      </c>
+      <c r="G29" s="73">
+        <v>46277</v>
+      </c>
+      <c r="H29" s="35"/>
+    </row>
+    <row r="30" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B30" t="s">
+        <v>204</v>
+      </c>
+      <c r="E30" s="82">
+        <f ca="1">NOW()</f>
+        <v>46277.53387835648</v>
+      </c>
+      <c r="G30" s="74">
+        <v>0.49722222222222223</v>
+      </c>
+    </row>
+    <row r="32" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="G32" t="s">
+        <v>224</v>
+      </c>
+      <c r="H32" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="33" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B33" s="85" t="s">
+        <v>211</v>
+      </c>
+      <c r="C33" s="85"/>
+      <c r="G33" t="s">
+        <v>222</v>
+      </c>
+      <c r="H33" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="34" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B34" s="85"/>
+      <c r="C34" s="85"/>
+      <c r="D34" t="s">
+        <v>212</v>
+      </c>
+      <c r="G34" t="s">
+        <v>221</v>
+      </c>
+      <c r="H34">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="35" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B35" t="s">
+        <v>268</v>
+      </c>
+      <c r="E35" s="82"/>
+      <c r="G35" t="s">
+        <v>215</v>
+      </c>
+      <c r="H35" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="36" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="D36" s="35" t="s">
+        <v>214</v>
+      </c>
+      <c r="G36" t="s">
+        <v>219</v>
+      </c>
+      <c r="H36" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="39" spans="2:8" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C39" s="86"/>
+      <c r="D39" s="88" t="s">
+        <v>213</v>
+      </c>
+      <c r="E39" s="68" t="s">
+        <v>217</v>
+      </c>
+      <c r="F39" s="68" t="s">
+        <v>218</v>
+      </c>
+      <c r="G39" s="88" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="40" spans="2:8" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C40" s="87">
+        <v>45679.604166666664</v>
+      </c>
+      <c r="D40" s="87" t="str">
+        <f>TEXT(C40,"dd-mm-yyyy" )</f>
+        <v>22-01-2025</v>
+      </c>
+      <c r="E40" s="87" t="str">
+        <f>TEXT(D40,"dd-mmm-yyyy" )</f>
+        <v>22-Jan-2025</v>
+      </c>
+      <c r="F40" s="87" t="str">
+        <f>TEXT(E40,"dd-mmmm-yyyy" )</f>
+        <v>22-January-2025</v>
+      </c>
+      <c r="G40" s="87" t="str">
+        <f>TEXT(C40,"hh:mm:ss" )</f>
+        <v>14:30:00</v>
+      </c>
+    </row>
+    <row r="41" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="C41" s="87">
+        <v>44561.34375</v>
+      </c>
+      <c r="D41" s="87" t="str">
+        <f>TEXT(C41,"dd-mm-yyyy" )</f>
+        <v>31-12-2021</v>
+      </c>
+      <c r="E41" s="87" t="str">
+        <f t="shared" ref="E41:F42" si="0">TEXT(D41,"dd-mmm-yyyy" )</f>
+        <v>31-Dec-2021</v>
+      </c>
+      <c r="F41" s="87" t="str">
+        <f t="shared" ref="F41:F42" si="1">TEXT(E41,"dd-mmmm-yyyy" )</f>
+        <v>31-December-2021</v>
+      </c>
+      <c r="G41" s="86"/>
+    </row>
+    <row r="42" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="C42" s="87">
+        <v>45056.781597222223</v>
+      </c>
+      <c r="D42" s="87" t="str">
+        <f t="shared" ref="D41:E42" si="2">TEXT(C42,"dd-mm-yyyy" )</f>
+        <v>10-05-2023</v>
+      </c>
+      <c r="E42" s="87" t="str">
+        <f t="shared" si="0"/>
+        <v>10-May-2023</v>
+      </c>
+      <c r="F42" s="87" t="str">
+        <f t="shared" si="1"/>
+        <v>10-May-2023</v>
+      </c>
+      <c r="G42" s="86"/>
+    </row>
+    <row r="45" spans="2:8" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C45" s="89">
+        <f ca="1">NOW()</f>
+        <v>46277.53387835648</v>
+      </c>
+      <c r="E45" s="34" t="str">
+        <f ca="1">TEXT(C45,"hh:mm:ss" )</f>
+        <v>12:48:47</v>
+      </c>
+    </row>
+    <row r="46" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="D46" t="s">
+        <v>229</v>
+      </c>
+      <c r="E46">
+        <f ca="1">HOUR(C45)</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="47" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="D47" t="s">
+        <v>230</v>
+      </c>
+      <c r="E47">
+        <f ca="1">MINUTE(C45)</f>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="48" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="D48" t="s">
+        <v>231</v>
+      </c>
+      <c r="E48">
+        <f ca="1">DAY(C45)</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="51" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C51" s="96" t="str">
+        <f ca="1" xml:space="preserve"> "Today is "         &amp;          TEXT(TODAY(),"dddd, mmmm dd, yyyy")       &amp;         " and the current time is "      &amp;TEXT(NOW(),"hh:mm:ss AM/PM")</f>
+        <v>Today is Saturday, September 12, 2026 and the current time is 12:48:47 PM</v>
+      </c>
+    </row>
+    <row r="53" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C53" s="32" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="54" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="D54" s="93" t="s">
+        <v>265</v>
+      </c>
+      <c r="F54" s="93" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="56" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B56" s="59" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="57" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C57" s="92" t="s">
+        <v>240</v>
+      </c>
+      <c r="D57" s="92"/>
+      <c r="E57" s="92"/>
+    </row>
+    <row r="58" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="C58" s="86"/>
+      <c r="D58" s="68" t="s">
+        <v>238</v>
+      </c>
+      <c r="E58" s="88" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="59" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C59" s="67" t="s">
+        <v>233</v>
+      </c>
+      <c r="D59" s="90">
+        <v>46308</v>
+      </c>
+      <c r="E59" s="91">
+        <f ca="1" xml:space="preserve"> D59 - TODAY()</f>
+        <v>31</v>
+      </c>
+      <c r="F59" s="35" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="60" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C60" s="67" t="s">
+        <v>234</v>
+      </c>
+      <c r="D60" s="90">
+        <v>46370</v>
+      </c>
+      <c r="E60" s="91">
+        <f t="shared" ref="E60:E63" ca="1" si="3" xml:space="preserve"> D60 - TODAY()</f>
+        <v>93</v>
+      </c>
+    </row>
+    <row r="61" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="C61" s="67" t="s">
+        <v>235</v>
+      </c>
+      <c r="D61" s="90">
+        <v>46341</v>
+      </c>
+      <c r="E61" s="91">
+        <f t="shared" ca="1" si="3"/>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="62" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B62" s="35"/>
+      <c r="C62" s="67" t="s">
+        <v>236</v>
+      </c>
+      <c r="D62" s="90">
+        <v>46342</v>
+      </c>
+      <c r="E62" s="91">
+        <f t="shared" ca="1" si="3"/>
+        <v>65</v>
+      </c>
+      <c r="F62" s="35"/>
+    </row>
+    <row r="63" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B63" s="35"/>
+      <c r="C63" s="67" t="s">
+        <v>237</v>
+      </c>
+      <c r="D63" s="90">
+        <v>46282</v>
+      </c>
+      <c r="E63" s="91">
+        <f t="shared" ca="1" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="F63" s="35"/>
+    </row>
+    <row r="64" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B64" s="35"/>
+      <c r="C64" s="35"/>
+      <c r="D64" s="35"/>
+      <c r="E64" s="35"/>
+      <c r="F64" s="35"/>
+    </row>
+    <row r="65" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B65" s="35"/>
+      <c r="C65" s="35"/>
+      <c r="D65" s="35"/>
+      <c r="E65" s="35"/>
+      <c r="F65" s="35"/>
+    </row>
+    <row r="66" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B66" s="35" t="s">
+        <v>232</v>
+      </c>
+      <c r="C66" s="35"/>
+      <c r="D66" s="35"/>
+      <c r="E66" s="35"/>
+      <c r="F66" s="35"/>
+    </row>
+    <row r="67" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B67" s="35"/>
+      <c r="C67" s="95" t="s">
+        <v>242</v>
+      </c>
+      <c r="D67" s="95"/>
+      <c r="E67" s="95"/>
+      <c r="F67" s="35"/>
+    </row>
+    <row r="68" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B68" s="35"/>
+      <c r="C68" s="84" t="s">
+        <v>24</v>
+      </c>
+      <c r="D68" s="84" t="s">
+        <v>246</v>
+      </c>
+      <c r="E68" s="84" t="s">
+        <v>247</v>
+      </c>
+      <c r="F68" s="35"/>
+    </row>
+    <row r="69" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B69" s="35"/>
+      <c r="C69" s="35" t="s">
+        <v>65</v>
+      </c>
+      <c r="D69" s="83">
+        <v>33008</v>
+      </c>
+      <c r="E69" s="36">
+        <f ca="1">DATEDIF(D69,TODAY(), "Y")</f>
+        <v>36</v>
+      </c>
+      <c r="F69" s="94" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="70" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B70" s="35"/>
+      <c r="C70" s="35" t="s">
+        <v>243</v>
+      </c>
+      <c r="D70" s="83">
+        <v>35201</v>
+      </c>
+      <c r="E70" s="36">
+        <f t="shared" ref="E70:E72" ca="1" si="4">DATEDIF(D70,TODAY(), "Y")</f>
+        <v>30</v>
+      </c>
+      <c r="F70" s="35"/>
+    </row>
+    <row r="71" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B71" s="35"/>
+      <c r="C71" s="35" t="s">
+        <v>244</v>
+      </c>
+      <c r="D71" s="83">
+        <v>35932</v>
+      </c>
+      <c r="E71" s="36">
+        <f t="shared" ca="1" si="4"/>
+        <v>28</v>
+      </c>
+      <c r="F71" s="35"/>
+    </row>
+    <row r="72" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B72" s="35"/>
+      <c r="C72" s="35" t="s">
+        <v>245</v>
+      </c>
+      <c r="D72" s="83">
+        <v>36664</v>
+      </c>
+      <c r="E72" s="36">
+        <f ca="1">DATEDIF(D72,TODAY(), "Y")</f>
+        <v>26</v>
+      </c>
+      <c r="F72" s="35"/>
+    </row>
+    <row r="73" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B73" s="35"/>
+      <c r="C73" s="35"/>
+      <c r="D73" s="35"/>
+      <c r="E73" s="35"/>
+      <c r="F73" s="35"/>
+    </row>
+    <row r="74" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B74" s="35"/>
+      <c r="C74" s="35"/>
+      <c r="D74" s="35"/>
+      <c r="E74" s="35"/>
+      <c r="F74" s="35"/>
+    </row>
+    <row r="75" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B75" s="59" t="s">
+        <v>248</v>
+      </c>
+      <c r="C75" s="35"/>
+      <c r="D75" s="35"/>
+      <c r="E75" s="35"/>
+      <c r="F75" s="35"/>
+    </row>
+    <row r="76" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B76" s="35"/>
+      <c r="C76" s="35" t="s">
+        <v>249</v>
+      </c>
+      <c r="D76" s="35"/>
+      <c r="E76" s="34">
+        <f xml:space="preserve"> DATEDIF("1/1/2026","12/09/2026","D")</f>
+        <v>254</v>
+      </c>
+      <c r="F76" s="94" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="77" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B77" s="35"/>
+      <c r="C77" s="35"/>
+      <c r="D77" s="35"/>
+      <c r="E77" s="35"/>
+      <c r="F77" s="35"/>
+    </row>
+    <row r="78" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B78" s="35"/>
+      <c r="C78" s="34" t="s">
+        <v>250</v>
+      </c>
+      <c r="D78" s="35"/>
+      <c r="E78" s="35"/>
+      <c r="F78" s="35"/>
+    </row>
+    <row r="79" spans="2:6" ht="16.8" x14ac:dyDescent="0.4">
+      <c r="B79" s="35"/>
+      <c r="C79" s="24" t="s">
+        <v>251</v>
+      </c>
+      <c r="D79" s="35" t="s">
+        <v>257</v>
+      </c>
+      <c r="E79" s="35"/>
+      <c r="F79" s="79"/>
+    </row>
+    <row r="80" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B80" s="35"/>
+      <c r="C80" s="24" t="s">
+        <v>252</v>
+      </c>
+      <c r="D80" s="35" t="s">
+        <v>258</v>
+      </c>
+      <c r="E80" s="35"/>
+      <c r="F80" s="35"/>
+    </row>
+    <row r="81" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B81" s="35"/>
+      <c r="C81" s="24" t="s">
+        <v>256</v>
+      </c>
+      <c r="D81" s="35" t="s">
+        <v>259</v>
+      </c>
+      <c r="E81" s="35"/>
+      <c r="F81" s="35"/>
+    </row>
+    <row r="82" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B82" s="35"/>
+      <c r="C82" s="24" t="s">
+        <v>255</v>
+      </c>
+      <c r="D82" s="35" t="s">
+        <v>260</v>
+      </c>
+      <c r="E82" s="35"/>
+      <c r="F82" s="35"/>
+    </row>
+    <row r="83" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B83" s="35"/>
+      <c r="C83" s="24" t="s">
+        <v>254</v>
+      </c>
+      <c r="D83" s="35" t="s">
+        <v>261</v>
+      </c>
+      <c r="E83" s="35"/>
+      <c r="F83" s="35"/>
+    </row>
+    <row r="84" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B84" s="35"/>
+      <c r="C84" s="24" t="s">
+        <v>253</v>
+      </c>
+      <c r="D84" s="35" t="s">
+        <v>262</v>
+      </c>
+      <c r="E84" s="35"/>
+      <c r="F84" s="35"/>
+    </row>
+    <row r="85" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B85" s="35"/>
+      <c r="C85" s="35"/>
+      <c r="D85" s="35"/>
+      <c r="E85" s="35"/>
+      <c r="F85" s="35"/>
+    </row>
+    <row r="86" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B86" s="35"/>
+      <c r="C86" s="35"/>
+      <c r="D86" s="35"/>
+      <c r="E86" s="35"/>
+      <c r="F86" s="35"/>
+    </row>
+    <row r="87" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B87" s="35"/>
+      <c r="C87" s="35"/>
+      <c r="D87" s="35"/>
+      <c r="E87" s="35"/>
+      <c r="F87" s="35"/>
+    </row>
+    <row r="88" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B88" s="35"/>
+      <c r="C88" s="35" t="s">
+        <v>269</v>
+      </c>
+      <c r="D88" s="35"/>
+      <c r="E88" s="35" t="s">
+        <v>270</v>
+      </c>
+      <c r="F88" s="35"/>
+    </row>
+    <row r="89" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B89" s="35"/>
+      <c r="C89" s="35"/>
+      <c r="D89" s="35"/>
+      <c r="E89" s="35" t="s">
+        <v>271</v>
+      </c>
+      <c r="F89" s="35"/>
+    </row>
+    <row r="90" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B90" s="35"/>
+      <c r="C90" s="35" t="s">
+        <v>272</v>
+      </c>
+      <c r="D90" s="35"/>
+      <c r="E90" s="35"/>
+      <c r="F90" s="35"/>
+    </row>
+    <row r="91" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B91" s="35"/>
+      <c r="C91" s="35"/>
+      <c r="D91" s="35"/>
+      <c r="E91" s="35"/>
+      <c r="F91" s="35"/>
+    </row>
+    <row r="92" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B92" s="35"/>
+      <c r="E92" s="35"/>
+      <c r="F92" s="35"/>
+    </row>
+    <row r="93" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B93" s="35"/>
+      <c r="C93" s="35"/>
+      <c r="D93" s="35" t="s">
+        <v>273</v>
+      </c>
+      <c r="E93" s="35"/>
+      <c r="F93" s="35"/>
+    </row>
+    <row r="94" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B94" s="35"/>
+      <c r="C94" s="83">
+        <v>46277</v>
+      </c>
+      <c r="D94" s="73">
+        <f>WORKDAY(C94, 10, {"24/09/2026","28/09/2026"})</f>
+        <v>46294</v>
+      </c>
+      <c r="E94" s="35"/>
+      <c r="F94" s="35"/>
+    </row>
+    <row r="95" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B95" s="35"/>
+      <c r="C95" s="35"/>
+      <c r="D95" s="35"/>
+      <c r="E95" s="35" t="s">
+        <v>274</v>
+      </c>
+      <c r="F95" s="35"/>
+    </row>
+    <row r="96" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B96" s="35"/>
+      <c r="C96" s="35"/>
+      <c r="D96" s="35"/>
+      <c r="E96" s="35"/>
+      <c r="F96" s="35" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="97" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B97" s="35"/>
+      <c r="C97" s="35"/>
+      <c r="D97" s="35"/>
+      <c r="E97" s="35"/>
+      <c r="F97" s="35" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="98" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B98" s="35"/>
+      <c r="C98" s="35"/>
+      <c r="D98" s="35"/>
+      <c r="E98" s="35"/>
+      <c r="F98" s="35"/>
+    </row>
+    <row r="99" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B99" s="35"/>
+      <c r="C99" s="35"/>
+      <c r="D99" s="35"/>
+      <c r="E99" s="35"/>
+      <c r="F99" s="35"/>
+    </row>
+    <row r="100" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B100" s="35"/>
+      <c r="C100" s="35"/>
+      <c r="D100" s="35"/>
+      <c r="E100" s="35"/>
+      <c r="F100" s="35"/>
+    </row>
+    <row r="101" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B101" s="35"/>
+      <c r="C101" s="35"/>
+      <c r="D101" s="35"/>
+      <c r="E101" s="35"/>
+      <c r="F101" s="35"/>
+    </row>
+    <row r="102" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B102" s="35"/>
+      <c r="C102" s="35"/>
+      <c r="D102" s="35"/>
+      <c r="E102" s="35"/>
+      <c r="F102" s="35"/>
+    </row>
+    <row r="103" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B103" s="35"/>
+      <c r="C103" s="35"/>
+      <c r="D103" s="35"/>
+      <c r="E103" s="35"/>
+      <c r="F103" s="35"/>
+    </row>
+    <row r="104" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B104" s="35"/>
+      <c r="C104" s="35"/>
+      <c r="D104" s="35"/>
+      <c r="E104" s="35"/>
+      <c r="F104" s="35"/>
+    </row>
+    <row r="105" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B105" s="35"/>
+      <c r="C105" s="35"/>
+      <c r="D105" s="35"/>
+      <c r="E105" s="35"/>
+      <c r="F105" s="35"/>
+    </row>
+    <row r="106" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B106" s="35"/>
+      <c r="C106" s="35"/>
+      <c r="D106" s="35"/>
+      <c r="E106" s="35"/>
+      <c r="F106" s="35"/>
+    </row>
+    <row r="107" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B107" s="35"/>
+      <c r="C107" s="35"/>
+      <c r="D107" s="35"/>
+      <c r="E107" s="35"/>
+      <c r="F107" s="35"/>
+    </row>
+    <row r="108" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B108" s="35"/>
+      <c r="C108" s="35"/>
+      <c r="D108" s="35"/>
+      <c r="E108" s="35"/>
+      <c r="F108" s="35"/>
+    </row>
+    <row r="109" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B109" s="35"/>
+      <c r="C109" s="35"/>
+      <c r="D109" s="35"/>
+      <c r="E109" s="35"/>
+      <c r="F109" s="35"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="C57:E57"/>
+    <mergeCell ref="B3:E4"/>
+    <mergeCell ref="B33:C34"/>
+  </mergeCells>
+  <phoneticPr fontId="27" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>